<commit_message>
Update NSE market report
</commit_message>
<xml_diff>
--- a/NSE_MARKET_REPORT/output/excel/NSE_Market_Report.xlsx
+++ b/NSE_MARKET_REPORT/output/excel/NSE_Market_Report.xlsx
@@ -11,8 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Losers" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Gainers'!$A$1:$O$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Losers'!$A$1:$O$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Gainers'!$A$1:$O$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Losers'!$A$1:$O$41</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O21"/>
+  <dimension ref="A1:O41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -577,7 +577,6 @@
       <c r="L2" t="n">
         <v>20</v>
       </c>
-      <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr">
         <is>
           <t>[]</t>
@@ -695,7 +694,6 @@
       <c r="L4" t="n">
         <v>20</v>
       </c>
-      <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr">
         <is>
           <t>[]</t>
@@ -996,7 +994,6 @@
       <c r="L9" t="n">
         <v>13.58</v>
       </c>
-      <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr">
         <is>
           <t>[]</t>
@@ -1419,7 +1416,6 @@
       <c r="L16" t="n">
         <v>9.99</v>
       </c>
-      <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr">
         <is>
           <t>[]</t>
@@ -1476,7 +1472,6 @@
       <c r="L17" t="n">
         <v>9.99</v>
       </c>
-      <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr">
         <is>
           <t>[]</t>
@@ -1655,7 +1650,6 @@
       <c r="L20" t="n">
         <v>9.609999999999999</v>
       </c>
-      <c r="M20" t="inlineStr"/>
       <c r="N20" t="inlineStr">
         <is>
           <t>[]</t>
@@ -1728,8 +1722,1216 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-08-14 10:19:04 IST</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Gainer</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>TECHNOCRAF</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Technocraft Ventures Limited</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>317.68</v>
+      </c>
+      <c r="F22" t="n">
+        <v>284</v>
+      </c>
+      <c r="G22" t="n">
+        <v>318</v>
+      </c>
+      <c r="H22" t="n">
+        <v>284</v>
+      </c>
+      <c r="I22" t="n">
+        <v>212</v>
+      </c>
+      <c r="J22" t="n">
+        <v>317.68</v>
+      </c>
+      <c r="K22" t="n">
+        <v>12239375</v>
+      </c>
+      <c r="L22" t="n">
+        <v>49.85</v>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>Technocraft Ventures Ltd. Share Price Today - Technocraft Ventures Ltd. Stock Price Live NSE/BSE - cnbctv18.com</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>['Technocraft Ventures Ltd. Share Price Today - Technocraft Ventures Ltd. Stock Price Live NSE/BSE - cnbctv18.com', 'Technocraft Ventures IPO Allotment Status: How to check share allotment online on NSE, BSE - Zee Business', 'Technocraft Ventures Limited: Performance &amp; Quotes, TECHNOCRAF Stock Price on NSE India S.E. Exchange - marketscreener.com', 'Technocraft Ventures IPO allotment status: How to check online on NSE, BSE, KFin Technologies - Dailyhunt', 'IPO Review: Technocraft Ventures Limited - moneylife.in']</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>AI remarks unavailable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-08-14 10:19:04 IST</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Gainer</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>BI</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Bilcare Limited</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>76.81</v>
+      </c>
+      <c r="F23" t="n">
+        <v>69.94</v>
+      </c>
+      <c r="G23" t="n">
+        <v>76.81</v>
+      </c>
+      <c r="H23" t="n">
+        <v>68.5</v>
+      </c>
+      <c r="I23" t="n">
+        <v>64.01000000000001</v>
+      </c>
+      <c r="J23" t="n">
+        <v>76.81</v>
+      </c>
+      <c r="K23" t="n">
+        <v>107009</v>
+      </c>
+      <c r="L23" t="n">
+        <v>20</v>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>【4901.T FY2026 Q1 Earnings Call】Bio CDMO Losses Balloon to ¥70 Billion, BI Partial IPO Planned; Revenue Hits Record on Semiconductor Materials but Operating Profit Slides 32% - finance.biggo.com</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>['【4901.T FY2026 Q1 Earnings Call】Bio CDMO Losses Balloon to ¥70 Billion, BI Partial IPO Planned; Revenue Hits Record on Semiconductor Materials but Operating Profit Slides 32% - finance.biggo.com', 'Bilcare Limited Announces Winding Up of Bilcare INC, A Wholly Owned Subsidiary of the Company - marketscreener.com', 'China’s CSI 300 Set to Lose Appeal Before Adding CXMT, BI Says - Bloomberg.com', "What AI-native analytics startups offer that BI vendors don't - techtarget.com", 'Shein IPO Value to Fall Short of $30 Billion Targeted by Some Investors, BI Says - Bloomberg.com']</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>AI remarks unavailable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-08-14 10:19:04 IST</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Gainer</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>APEX</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Apex Frozen Foods Limited</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>441.2</v>
+      </c>
+      <c r="F24" t="n">
+        <v>425.1</v>
+      </c>
+      <c r="G24" t="n">
+        <v>441.2</v>
+      </c>
+      <c r="H24" t="n">
+        <v>403.15</v>
+      </c>
+      <c r="I24" t="n">
+        <v>367.7</v>
+      </c>
+      <c r="J24" t="n">
+        <v>441.2</v>
+      </c>
+      <c r="K24" t="n">
+        <v>4696738</v>
+      </c>
+      <c r="L24" t="n">
+        <v>19.99</v>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>Apex Treasury Corporation Reports Earnings Results for the Second Quarter and Six Months Ended June 30, 2026 - marketscreener.com</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>['Apex Treasury Corporation Reports Earnings Results for the Second Quarter and Six Months Ended June 30, 2026 - marketscreener.com', 'Apex Biotechnology Corp. Reports Earnings Results for the Second Quarter and Six Months Ended June 30, 2026 - marketscreener.com', 'Maha Rashtra Apex Q1 Results: Consolidated profit up 85% YoY to ₹347.6 lakh - scanx.trade', 'Apex Capital &amp; Finance Q1 Results: Net profit rises 74% YoY - scanx.trade', 'Apex Capital and Finance Q1 Results: Net profit rises 73% YoY - scanx.trade']</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>AI remarks unavailable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-08-14 10:19:04 IST</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Gainer</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>OSWALSEEDS</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>ShreeOswal Seeds And Chemicals Limited</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>12.15</v>
+      </c>
+      <c r="F25" t="n">
+        <v>11.79</v>
+      </c>
+      <c r="G25" t="n">
+        <v>12.15</v>
+      </c>
+      <c r="H25" t="n">
+        <v>11</v>
+      </c>
+      <c r="I25" t="n">
+        <v>10.13</v>
+      </c>
+      <c r="J25" t="n">
+        <v>12.15</v>
+      </c>
+      <c r="K25" t="n">
+        <v>913586</v>
+      </c>
+      <c r="L25" t="n">
+        <v>19.94</v>
+      </c>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>AI remarks unavailable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-08-14 10:19:04 IST</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Gainer</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>TPHQ</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Teamo Productions HQ Limited</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="I26" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="J26" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="K26" t="n">
+        <v>8163583</v>
+      </c>
+      <c r="L26" t="n">
+        <v>19.51</v>
+      </c>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>AI remarks unavailable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-08-14 10:19:04 IST</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Gainer</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>GALAXYSURF</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Galaxy Surfactants Limited</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>2497.8</v>
+      </c>
+      <c r="F27" t="n">
+        <v>2412.5</v>
+      </c>
+      <c r="G27" t="n">
+        <v>2508.4</v>
+      </c>
+      <c r="H27" t="n">
+        <v>2391.2</v>
+      </c>
+      <c r="I27" t="n">
+        <v>2090.4</v>
+      </c>
+      <c r="J27" t="n">
+        <v>2497.8</v>
+      </c>
+      <c r="K27" t="n">
+        <v>434720</v>
+      </c>
+      <c r="L27" t="n">
+        <v>19.49</v>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>Galaxy Surfactants approves ₹22 final dividend at 40th AGM - scanx.trade</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>['Galaxy Surfactants approves ₹22 final dividend at 40th AGM - scanx.trade']</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>AI remarks unavailable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-08-14 10:19:04 IST</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Gainer</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>MANORAMA</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Manorama Industries Limited</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>1861</v>
+      </c>
+      <c r="F28" t="n">
+        <v>1729</v>
+      </c>
+      <c r="G28" t="n">
+        <v>1868</v>
+      </c>
+      <c r="H28" t="n">
+        <v>1683.1</v>
+      </c>
+      <c r="I28" t="n">
+        <v>1614.1</v>
+      </c>
+      <c r="J28" t="n">
+        <v>1861</v>
+      </c>
+      <c r="K28" t="n">
+        <v>2704746</v>
+      </c>
+      <c r="L28" t="n">
+        <v>15.3</v>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>Manorama Industries: Final Dividend Record Date Announced - InvestyWise</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>['Manorama Industries: Final Dividend Record Date Announced - InvestyWise', 'MANORAMA: Q1FY27 revenue up 39.5% YoY, PAT up 67.6% YoY, with strong global expansion and capex plans - TradingView', 'What is ‘One Herb, One Standard initiative’? - Manorama Yearbook', 'National Commission for Scheduled Castes submits annual report to President Murmu - Manorama Yearbook', 'Congo’s Ebola outbreak set to become deadliest on record, warns WHO - Manorama Yearbook']</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>AI remarks unavailable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-08-14 10:19:04 IST</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Gainer</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>HMAAGRO</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>HMA Agro Industries Limited</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>25.08</v>
+      </c>
+      <c r="F29" t="n">
+        <v>23</v>
+      </c>
+      <c r="G29" t="n">
+        <v>25.34</v>
+      </c>
+      <c r="H29" t="n">
+        <v>22</v>
+      </c>
+      <c r="I29" t="n">
+        <v>21.91</v>
+      </c>
+      <c r="J29" t="n">
+        <v>25.08</v>
+      </c>
+      <c r="K29" t="n">
+        <v>5532483</v>
+      </c>
+      <c r="L29" t="n">
+        <v>14.47</v>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>HMA Agro Industries Q1 Results: Earnings Call Scheduled for Aug 14 - scanx.trade</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>['HMA Agro Industries Q1 Results: Earnings Call Scheduled for Aug 14 - scanx.trade', 'HMA Agro Industries reports ₹21,103.19 million revenue for Q1 FY 2026-2027 - Business Upturn', 'HMA Agro Publishes Investor Presentation for June 2026 Quarter - tipranks.com', 'HMA Agro Industries Releases Q1 FY2026 Investor Presentation - tipranks.com']</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>AI remarks unavailable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-08-14 10:19:04 IST</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Gainer</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>LPDC</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Landmark Property Development Company Limited</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>8.65</v>
+      </c>
+      <c r="F30" t="n">
+        <v>8.619999999999999</v>
+      </c>
+      <c r="G30" t="n">
+        <v>9.050000000000001</v>
+      </c>
+      <c r="H30" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="I30" t="n">
+        <v>7.56</v>
+      </c>
+      <c r="J30" t="n">
+        <v>8.65</v>
+      </c>
+      <c r="K30" t="n">
+        <v>1007660</v>
+      </c>
+      <c r="L30" t="n">
+        <v>14.42</v>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>Gadzama to Rely on 2015 NBA Clearance in Appeal Against LPDC Suspension - Radio Nigeria Lagos</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>['Gadzama to Rely on 2015 NBA Clearance in Appeal Against LPDC Suspension - Radio Nigeria Lagos', 'LPDC Target Crowned Sarawak Closed Doubles Darts Champions - Sarawak Tribune', 'Zaki Biam Killings: LPDC Slams Three Years Suspension on Gadzama for Professional Misconduct - THISDAYLIVE', 'Full reasons why LPDC suspended senior advocate Gadzama, fellow lawyer from legal practice (DOWNLOAD) - Premium Times Nigeria', 'LPDC fixes Sept 30 for ruling in c’s alleged misconduct case - The Nation Newspaper']</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>AI remarks unavailable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-08-14 10:19:04 IST</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Gainer</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>XTRANET</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Xtranet Technologies Limited</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>168.17</v>
+      </c>
+      <c r="F31" t="n">
+        <v>148.5</v>
+      </c>
+      <c r="G31" t="n">
+        <v>170.3</v>
+      </c>
+      <c r="H31" t="n">
+        <v>148.5</v>
+      </c>
+      <c r="I31" t="n">
+        <v>150.4</v>
+      </c>
+      <c r="J31" t="n">
+        <v>168.17</v>
+      </c>
+      <c r="K31" t="n">
+        <v>737568</v>
+      </c>
+      <c r="L31" t="n">
+        <v>11.82</v>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>Xtranet Technologies IPO Lists At Premium On NSE And BSE - NDTV Profit</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>['Xtranet Technologies IPO Lists At Premium On NSE And BSE - NDTV Profit', 'Price to earnings ratio of Xtranet Technologies Limited – NSE:XTRANET - TradingView', 'Indo-MIM, Lohia Corp, Xtranet Technologies List At A Premium; Check Share Price - NDTV Profit', 'Xtranet Technologies Limited Revenue Breakdown – NSE:XTRANET - TradingView', 'Xtranet Technologies Limited Income Statement – NSE:XTRANET - TradingView']</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>AI remarks unavailable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-08-14 10:19:04 IST</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Gainer</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>BALUFORGE</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Balu Forge Industries Limited</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>493.4</v>
+      </c>
+      <c r="F32" t="n">
+        <v>450</v>
+      </c>
+      <c r="G32" t="n">
+        <v>503</v>
+      </c>
+      <c r="H32" t="n">
+        <v>449.15</v>
+      </c>
+      <c r="I32" t="n">
+        <v>446.25</v>
+      </c>
+      <c r="J32" t="n">
+        <v>493.4</v>
+      </c>
+      <c r="K32" t="n">
+        <v>3159579</v>
+      </c>
+      <c r="L32" t="n">
+        <v>10.57</v>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>Balu Forge Industries announces strong Q1 FY27 results with aerospace sector entry - Business Upturn</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>['Balu Forge Industries announces strong Q1 FY27 results with aerospace sector entry - Business Upturn', 'Balu Forge Industries Q1 FY27: Net Profit Rises 15.9% YoY; Board Approves $60 Million Fundraise - Trade Brains', 'Balu Forge Board Approves $60M FCCB Issue &amp; ₹1000Cr Borrowing Hike - InvestyWise']</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>AI remarks unavailable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-08-14 10:19:04 IST</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Gainer</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>WELSPUNLIV</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Welspun Living Limited</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>174.82</v>
+      </c>
+      <c r="F33" t="n">
+        <v>170</v>
+      </c>
+      <c r="G33" t="n">
+        <v>178</v>
+      </c>
+      <c r="H33" t="n">
+        <v>165.16</v>
+      </c>
+      <c r="I33" t="n">
+        <v>159.83</v>
+      </c>
+      <c r="J33" t="n">
+        <v>174.82</v>
+      </c>
+      <c r="K33" t="n">
+        <v>37599345</v>
+      </c>
+      <c r="L33" t="n">
+        <v>9.380000000000001</v>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>WELSPUNLIV Share Price Today - Welspun Living on NSE/BSE - scanx.trade</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>['WELSPUNLIV Share Price Today - Welspun Living on NSE/BSE - scanx.trade', 'Number of shareholders of Welspun Living Limited – NSE:WELSPUNLIV - TradingView', 'Earnings call transcript: Welspun Living lifts Q1 2026 sales, stock falls 3.3% - Investing.com India', 'Welspun Living: Strong Q1 FY27 Results with Revenue Up 23.5% - InvestyWise', 'Welspun Living: Q1 FY27 Revenue Jumps 23.5% to ₹2,828 Crore - InvestyWise']</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>AI remarks unavailable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-08-14 10:19:04 IST</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Gainer</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>ZEEMEDIA</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Zee Media Corporation Limited</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>9.369999999999999</v>
+      </c>
+      <c r="F34" t="n">
+        <v>9.390000000000001</v>
+      </c>
+      <c r="G34" t="n">
+        <v>9.73</v>
+      </c>
+      <c r="H34" t="n">
+        <v>8.880000000000001</v>
+      </c>
+      <c r="I34" t="n">
+        <v>8.58</v>
+      </c>
+      <c r="J34" t="n">
+        <v>9.369999999999999</v>
+      </c>
+      <c r="K34" t="n">
+        <v>26669502</v>
+      </c>
+      <c r="L34" t="n">
+        <v>9.210000000000001</v>
+      </c>
+      <c r="M34" t="inlineStr"/>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>AI remarks unavailable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-08-14 10:19:04 IST</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Gainer</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>ATAM</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Atam Valves Limited</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>59.25</v>
+      </c>
+      <c r="F35" t="n">
+        <v>54.8</v>
+      </c>
+      <c r="G35" t="n">
+        <v>59.95</v>
+      </c>
+      <c r="H35" t="n">
+        <v>54.53</v>
+      </c>
+      <c r="I35" t="n">
+        <v>54.35</v>
+      </c>
+      <c r="J35" t="n">
+        <v>59.25</v>
+      </c>
+      <c r="K35" t="n">
+        <v>44189</v>
+      </c>
+      <c r="L35" t="n">
+        <v>9.02</v>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>Atam Valves Q1 Results: Net profit falls 49% YoY to ₹63.5 lakh - scanx.trade</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>['Atam Valves Q1 Results: Net profit falls 49% YoY to ₹63.5 lakh - scanx.trade', 'Community Highlights: Meet Dunebari Atam of Blueprint Financial Firm &amp; EveryOneWins - voyagedallas.com']</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>AI remarks unavailable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-08-14 10:19:04 IST</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Gainer</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>TIIL</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Technocraft Industries (India) Limited</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>3136.2</v>
+      </c>
+      <c r="F36" t="n">
+        <v>3145</v>
+      </c>
+      <c r="G36" t="n">
+        <v>3299.9</v>
+      </c>
+      <c r="H36" t="n">
+        <v>3061.2</v>
+      </c>
+      <c r="I36" t="n">
+        <v>2887.6</v>
+      </c>
+      <c r="J36" t="n">
+        <v>3136.2</v>
+      </c>
+      <c r="K36" t="n">
+        <v>458617</v>
+      </c>
+      <c r="L36" t="n">
+        <v>8.609999999999999</v>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>Tiil Morning Airbus A380 (9GrJB881u0) - Mshale</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>['Tiil Morning Airbus A380 (9GrJB881u0) - Mshale']</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>AI remarks unavailable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-08-14 10:19:04 IST</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Gainer</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>ISFT</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Intrasoft Technologies Limited</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>83</v>
+      </c>
+      <c r="F37" t="n">
+        <v>77.89</v>
+      </c>
+      <c r="G37" t="n">
+        <v>84.5</v>
+      </c>
+      <c r="H37" t="n">
+        <v>77.89</v>
+      </c>
+      <c r="I37" t="n">
+        <v>76.70999999999999</v>
+      </c>
+      <c r="J37" t="n">
+        <v>83</v>
+      </c>
+      <c r="K37" t="n">
+        <v>14255</v>
+      </c>
+      <c r="L37" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>IntraSoft Technologies Limited (533181.BO) stock price, news, quote and history - Yahoo Finance UK</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>['IntraSoft Technologies Limited (533181.BO) stock price, news, quote and history - Yahoo Finance UK', 'Intrasoft Technologies Releases Q1 FY2026 Investor Presentation - tipranks.com']</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>AI remarks unavailable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-08-14 10:19:04 IST</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Gainer</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>LGEINDIA</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>LG Electronics India Limited</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>1701.8</v>
+      </c>
+      <c r="F38" t="n">
+        <v>1620</v>
+      </c>
+      <c r="G38" t="n">
+        <v>1704.7</v>
+      </c>
+      <c r="H38" t="n">
+        <v>1611</v>
+      </c>
+      <c r="I38" t="n">
+        <v>1578.3</v>
+      </c>
+      <c r="J38" t="n">
+        <v>1701.8</v>
+      </c>
+      <c r="K38" t="n">
+        <v>4442442</v>
+      </c>
+      <c r="L38" t="n">
+        <v>7.82</v>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>LG Electronics India Limited Reports Earnings Results for the First Quarter Ended June 30, 2026 - marketscreener.com</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>['LG Electronics India Limited Reports Earnings Results for the First Quarter Ended June 30, 2026 - marketscreener.com', 'LG Electronics India Q1 Results: Earnings call scheduled for Aug 14 - scanx.trade', "LG Electronics India's quarterly profit rises on strong summer appliance sales - marketscreener.com", 'LG Electronics India Posts Strongest Quarterly Growth Since Listing - tipranks.com']</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>AI remarks unavailable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-08-14 10:19:04 IST</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Gainer</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>AYMSYNTEX</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>AYM Syntex Limited</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>274.95</v>
+      </c>
+      <c r="F39" t="n">
+        <v>261.75</v>
+      </c>
+      <c r="G39" t="n">
+        <v>276.6</v>
+      </c>
+      <c r="H39" t="n">
+        <v>258</v>
+      </c>
+      <c r="I39" t="n">
+        <v>256.45</v>
+      </c>
+      <c r="J39" t="n">
+        <v>274.95</v>
+      </c>
+      <c r="K39" t="n">
+        <v>37857</v>
+      </c>
+      <c r="L39" t="n">
+        <v>7.21</v>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>AYM Syntex Limited Reports Earnings Results for the First Quarter Ended June 30, 2026 - marketscreener.com</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>['AYM Syntex Limited Reports Earnings Results for the First Quarter Ended June 30, 2026 - marketscreener.com']</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>AI remarks unavailable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-08-14 10:19:04 IST</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Gainer</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>JNKINDIA</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>JNK India Limited</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>441.75</v>
+      </c>
+      <c r="F40" t="n">
+        <v>429.85</v>
+      </c>
+      <c r="G40" t="n">
+        <v>449.95</v>
+      </c>
+      <c r="H40" t="n">
+        <v>425</v>
+      </c>
+      <c r="I40" t="n">
+        <v>413.15</v>
+      </c>
+      <c r="J40" t="n">
+        <v>441.75</v>
+      </c>
+      <c r="K40" t="n">
+        <v>551045</v>
+      </c>
+      <c r="L40" t="n">
+        <v>6.92</v>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>JNKINDIA: Revenue and profit surged in Q1 FY 2027, with strong order book and diversification underway - TradingView</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>['JNKINDIA: Revenue and profit surged in Q1 FY 2027, with strong order book and diversification underway - TradingView', 'JNKINDIA: Revenue up 80.6% YoY; order book at INR 1,801 cr; diversification on track - TradingView', 'JNKINDIA: Q1FY27 delivered 80.6% YoY income growth and robust margins, with strong order visibility - TradingView', 'JNK India Limited Reports Earnings Results for the First Quarter Ended June 30, 2026 - marketscreener.com', 'JNK India Q1 Results: Net profit surges 1,059% YoY to ₹96.25 million - scanx.trade']</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>AI remarks unavailable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-08-14 10:19:04 IST</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Gainer</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>MOTISONS</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Motisons Jewellers Limited</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>15.61</v>
+      </c>
+      <c r="F41" t="n">
+        <v>14.76</v>
+      </c>
+      <c r="G41" t="n">
+        <v>15.84</v>
+      </c>
+      <c r="H41" t="n">
+        <v>14.48</v>
+      </c>
+      <c r="I41" t="n">
+        <v>14.62</v>
+      </c>
+      <c r="J41" t="n">
+        <v>15.61</v>
+      </c>
+      <c r="K41" t="n">
+        <v>69267238</v>
+      </c>
+      <c r="L41" t="n">
+        <v>6.77</v>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>Motisons Jewellers Q1 Results: Net profit up 38% to ₹110.5 crore - scanx.trade</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>['Motisons Jewellers Q1 Results: Net profit up 38% to ₹110.5 crore - scanx.trade', "Motisons Jewellers shares jump 5% on heavy volumes after Q1 results: Here's what the numbers showed - Business Upturn", 'Motisons Jewellers standalone net profit rises 37.61% in the June 2026 quarter - business-standard.com', 'Motisons Jewellers Ltd Revenue Breakdown – NSE:MOTISONS - TradingView', 'Black Box shares jump over 7% after Q1 EBITDA rises 39% YoY to Rs 150 crore, revenue grows 24% - Business Upturn']</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>AI remarks unavailable.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O21"/>
+  <autoFilter ref="A1:O41"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1740,7 +2942,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O21"/>
+  <dimension ref="A1:O41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2248,7 +3450,6 @@
       <c r="L8" t="n">
         <v>-8.300000000000001</v>
       </c>
-      <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr">
         <is>
           <t>[]</t>
@@ -2488,7 +3689,6 @@
       <c r="L12" t="n">
         <v>-8.58</v>
       </c>
-      <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr">
         <is>
           <t>[]</t>
@@ -2911,7 +4111,6 @@
       <c r="L19" t="n">
         <v>-13.34</v>
       </c>
-      <c r="M19" t="inlineStr"/>
       <c r="N19" t="inlineStr">
         <is>
           <t>[]</t>
@@ -3045,8 +4244,1188 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-08-14 10:19:04 IST</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Loser</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>LEAPIND</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>LEAP India Limited</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>153.46</v>
+      </c>
+      <c r="F22" t="n">
+        <v>165.9</v>
+      </c>
+      <c r="G22" t="n">
+        <v>167</v>
+      </c>
+      <c r="H22" t="n">
+        <v>152.3</v>
+      </c>
+      <c r="I22" t="n">
+        <v>159</v>
+      </c>
+      <c r="J22" t="n">
+        <v>153.46</v>
+      </c>
+      <c r="K22" t="n">
+        <v>49822702</v>
+      </c>
+      <c r="L22" t="n">
+        <v>-3.48</v>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>Basic earnings per share (basic EPS) of LEAP India Limited – NSE:LEAP - TradingView</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>['Basic earnings per share (basic EPS) of LEAP India Limited – NSE:LEAP - TradingView', 'Operating margin % of LEAP India Limited – NSE:LEAP - TradingView', 'LEAP India Limited Revenue Breakdown – NSE:LEAP - TradingView', 'LEAP India Limited Balance Sheet – NSE:LEAP - TradingView', 'LEAP India Limited Cash Flow – NSE:LEAP - TradingView']</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>AI remarks unavailable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-08-14 10:19:04 IST</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Loser</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>TMPV</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Tata Motors Passenger Vehicles Limited</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>330.8</v>
+      </c>
+      <c r="F23" t="n">
+        <v>329</v>
+      </c>
+      <c r="G23" t="n">
+        <v>337.75</v>
+      </c>
+      <c r="H23" t="n">
+        <v>329</v>
+      </c>
+      <c r="I23" t="n">
+        <v>349.6</v>
+      </c>
+      <c r="J23" t="n">
+        <v>330.8</v>
+      </c>
+      <c r="K23" t="n">
+        <v>14687197</v>
+      </c>
+      <c r="L23" t="n">
+        <v>-5.38</v>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>Q1 Results 14th Aug Live: Anupam Rasayan PAT up marginally, Ashok Leyland, NMDC, Alkem Lab, Bharat Dynamics, Voltas, 3M India, Cochin Shipyard, Physicswallah, Cholamandalam Fin, PTC Ind, Natco Pharma, Borosil to announce Q1 results, TMPV, Ma - BusinessLine</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>['Q1 Results 14th Aug Live: Anupam Rasayan PAT up marginally, Ashok Leyland, NMDC, Alkem Lab, Bharat Dynamics, Voltas, 3M India, Cochin Shipyard, Physicswallah, Cholamandalam Fin, PTC Ind, Natco Pharma, Borosil to announce Q1 results, TMPV, Ma - BusinessLine', 'Q1 Results 13th Aug Live: TMPV, Solar Ind, LG Electronics, Max Healthcare, GIC, Godrej Ind, Jubilant Foodworks, Amber Enterprises, Indraprastha Gas, Brigade, JSW Cement, Honasa Consumer to announce Q1 results, Tata Motors, HAL, Apollo Hospitals, Gr - BusinessLine', 'TMPV shares fall nearly 6% as JLR weakness and margin concerns weigh, brokerages divided - BusinessLine', 'Stocks to watch: Honasa, LG Electronics, Physicswalla, NMDC, TMPV - business-standard.com', 'Remain fully focused on driving growth: TMPV amid imminent change in Tata Group leadership - The Hans India']</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>AI remarks unavailable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-08-14 10:19:04 IST</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Loser</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>ZOTA</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Zota Health Care LImited</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>1173.7</v>
+      </c>
+      <c r="F24" t="n">
+        <v>1231.3</v>
+      </c>
+      <c r="G24" t="n">
+        <v>1236.1</v>
+      </c>
+      <c r="H24" t="n">
+        <v>1163.2</v>
+      </c>
+      <c r="I24" t="n">
+        <v>1241.3</v>
+      </c>
+      <c r="J24" t="n">
+        <v>1173.7</v>
+      </c>
+      <c r="K24" t="n">
+        <v>79127</v>
+      </c>
+      <c r="L24" t="n">
+        <v>-5.45</v>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>Zota Health Care Ltd Says June-Quarter Consol Net Loss 435.6 Million Rupees - TradingView</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>['Zota Health Care Ltd Says June-Quarter Consol Net Loss 435.6 Million Rupees - TradingView', 'Q1 Results: Tata Motors PV, Solar Industries, LG Electronics, Max Healthcare, General Insurance, Page Industries, others to declare earnings on August 13 - Dailyhunt', 'Zota Health Care Ltd is Rated Strong Sell - MarketsMojo', 'Water and energy jobs push Costain to ‘inflection point’ - Construction News']</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>AI remarks unavailable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-08-14 10:19:04 IST</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Loser</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>VPRPL</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Vishnu Prakash R Punglia Limited</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>32.99</v>
+      </c>
+      <c r="F25" t="n">
+        <v>33.4</v>
+      </c>
+      <c r="G25" t="n">
+        <v>36</v>
+      </c>
+      <c r="H25" t="n">
+        <v>32.9</v>
+      </c>
+      <c r="I25" t="n">
+        <v>34.97</v>
+      </c>
+      <c r="J25" t="n">
+        <v>32.99</v>
+      </c>
+      <c r="K25" t="n">
+        <v>689181</v>
+      </c>
+      <c r="L25" t="n">
+        <v>-5.66</v>
+      </c>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>AI remarks unavailable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-08-14 10:19:04 IST</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Loser</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>GOCLCORP</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>GOCL Corporation Limited</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>405.8</v>
+      </c>
+      <c r="F26" t="n">
+        <v>417.55</v>
+      </c>
+      <c r="G26" t="n">
+        <v>418.1</v>
+      </c>
+      <c r="H26" t="n">
+        <v>403.85</v>
+      </c>
+      <c r="I26" t="n">
+        <v>430.9</v>
+      </c>
+      <c r="J26" t="n">
+        <v>405.8</v>
+      </c>
+      <c r="K26" t="n">
+        <v>59961</v>
+      </c>
+      <c r="L26" t="n">
+        <v>-5.83</v>
+      </c>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>AI remarks unavailable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-08-14 10:19:04 IST</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Loser</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>SWELECTES</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Swelect Energy Systems Limited</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>639.3</v>
+      </c>
+      <c r="F27" t="n">
+        <v>663</v>
+      </c>
+      <c r="G27" t="n">
+        <v>667.95</v>
+      </c>
+      <c r="H27" t="n">
+        <v>625</v>
+      </c>
+      <c r="I27" t="n">
+        <v>681.25</v>
+      </c>
+      <c r="J27" t="n">
+        <v>639.3</v>
+      </c>
+      <c r="K27" t="n">
+        <v>43507</v>
+      </c>
+      <c r="L27" t="n">
+        <v>-6.16</v>
+      </c>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>AI remarks unavailable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-08-14 10:19:04 IST</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Loser</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>MIDHANI</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Mishra Dhatu Nigam Limited</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>417.35</v>
+      </c>
+      <c r="F28" t="n">
+        <v>444</v>
+      </c>
+      <c r="G28" t="n">
+        <v>447.7</v>
+      </c>
+      <c r="H28" t="n">
+        <v>415.1</v>
+      </c>
+      <c r="I28" t="n">
+        <v>444.85</v>
+      </c>
+      <c r="J28" t="n">
+        <v>417.35</v>
+      </c>
+      <c r="K28" t="n">
+        <v>2337306</v>
+      </c>
+      <c r="L28" t="n">
+        <v>-6.18</v>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>Midhani Q1 results: net profit up 27%, EBITDA margin narrows - Business Upturn</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>['Midhani Q1 results: net profit up 27%, EBITDA margin narrows - Business Upturn', 'MIDHANI: Q1 FY27 Results Show Strong Growth - InvestyWise', 'MIDHANI Shares Hit 52-Week High After GE Aerospace S400 Nod - Whalesbook', 'Why MIDHANI shares are rallying over 6% today? Here’s what triggered the rally - Business Upturn', 'MIDHANI becomes first Indian company to secure GE Aerospace S400 lab approval - cnbctv18.com']</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>AI remarks unavailable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-08-14 10:19:04 IST</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Loser</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>ARDEE</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Ardee Industries Limited</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>60.67</v>
+      </c>
+      <c r="F29" t="n">
+        <v>64.78</v>
+      </c>
+      <c r="G29" t="n">
+        <v>64.78</v>
+      </c>
+      <c r="H29" t="n">
+        <v>60.59</v>
+      </c>
+      <c r="I29" t="n">
+        <v>64.87</v>
+      </c>
+      <c r="J29" t="n">
+        <v>60.67</v>
+      </c>
+      <c r="K29" t="n">
+        <v>9546604</v>
+      </c>
+      <c r="L29" t="n">
+        <v>-6.47</v>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>Ardee Industries Limited Earnings and Revenue – BSE:ARDEE - TradingView</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>['Ardee Industries Limited Earnings and Revenue – BSE:ARDEE - TradingView', 'Price to earnings ratio of Ardee Industries Limited – BSE:ARDEE - TradingView', 'Gross profit of Ardee Industries Limited – BSE:ARDEE - TradingView', 'CapEx per share of Ardee Industries Limited – NSE:ARDEE - TradingView', 'Net margin % of Ardee Industries Limited – BSE:ARDEE - TradingView']</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>AI remarks unavailable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-08-14 10:19:04 IST</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Loser</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>FINOPB</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Fino Payments Bank Limited</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>152.42</v>
+      </c>
+      <c r="F30" t="n">
+        <v>158</v>
+      </c>
+      <c r="G30" t="n">
+        <v>158</v>
+      </c>
+      <c r="H30" t="n">
+        <v>150.53</v>
+      </c>
+      <c r="I30" t="n">
+        <v>163.7</v>
+      </c>
+      <c r="J30" t="n">
+        <v>152.42</v>
+      </c>
+      <c r="K30" t="n">
+        <v>627703</v>
+      </c>
+      <c r="L30" t="n">
+        <v>-6.89</v>
+      </c>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>AI remarks unavailable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-08-14 10:19:04 IST</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Loser</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>HARRMALAYA</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Harrisons Malayalam Limited</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>207</v>
+      </c>
+      <c r="F31" t="n">
+        <v>209.07</v>
+      </c>
+      <c r="G31" t="n">
+        <v>209.5</v>
+      </c>
+      <c r="H31" t="n">
+        <v>205</v>
+      </c>
+      <c r="I31" t="n">
+        <v>222.68</v>
+      </c>
+      <c r="J31" t="n">
+        <v>207</v>
+      </c>
+      <c r="K31" t="n">
+        <v>17461</v>
+      </c>
+      <c r="L31" t="n">
+        <v>-7.04</v>
+      </c>
+      <c r="M31" t="inlineStr"/>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>AI remarks unavailable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-08-14 10:19:04 IST</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Loser</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>GENESYS</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Genesys International Corporation Limited</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>196.4</v>
+      </c>
+      <c r="F32" t="n">
+        <v>209.45</v>
+      </c>
+      <c r="G32" t="n">
+        <v>211.3</v>
+      </c>
+      <c r="H32" t="n">
+        <v>195.9</v>
+      </c>
+      <c r="I32" t="n">
+        <v>211.3</v>
+      </c>
+      <c r="J32" t="n">
+        <v>196.4</v>
+      </c>
+      <c r="K32" t="n">
+        <v>282149</v>
+      </c>
+      <c r="L32" t="n">
+        <v>-7.05</v>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>Lawsuit filed against former Genesys doctor, hospital - MLive.com</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>['Lawsuit filed against former Genesys doctor, hospital - MLive.com', '2026-2027 YCS Advanced &amp; Genesys Prizing - ygorganization.com', 'Lawsuit filed against former Genesys doctor, hospital - NewsBreak: Local News &amp; Alerts', 'Genesys Puts AI Trust at the Center of Its Agentic CX Strategy - CX Today', 'Genesys’ Impact: Sustainable Procurement &amp; Responsible AI - Sustainability Magazine']</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>AI remarks unavailable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-08-14 10:19:04 IST</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Loser</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>MAHAPEXLTD</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Maha Rashtra Apex Corporation Limited</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>50.86</v>
+      </c>
+      <c r="F33" t="n">
+        <v>53.8</v>
+      </c>
+      <c r="G33" t="n">
+        <v>53.8</v>
+      </c>
+      <c r="H33" t="n">
+        <v>49.35</v>
+      </c>
+      <c r="I33" t="n">
+        <v>54.74</v>
+      </c>
+      <c r="J33" t="n">
+        <v>50.86</v>
+      </c>
+      <c r="K33" t="n">
+        <v>42944</v>
+      </c>
+      <c r="L33" t="n">
+        <v>-7.09</v>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>Maha Rashtra Apex signs deal to market Paulownia timber in India - scanx.trade</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>['Maha Rashtra Apex signs deal to market Paulownia timber in India - scanx.trade']</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>AI remarks unavailable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-08-14 10:19:04 IST</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Loser</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>BELLACASA</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Bella Casa Fashion &amp; Retail Limited</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>221</v>
+      </c>
+      <c r="F34" t="n">
+        <v>237.39</v>
+      </c>
+      <c r="G34" t="n">
+        <v>237.4</v>
+      </c>
+      <c r="H34" t="n">
+        <v>220.2</v>
+      </c>
+      <c r="I34" t="n">
+        <v>239.51</v>
+      </c>
+      <c r="J34" t="n">
+        <v>221</v>
+      </c>
+      <c r="K34" t="n">
+        <v>19320</v>
+      </c>
+      <c r="L34" t="n">
+        <v>-7.73</v>
+      </c>
+      <c r="M34" t="inlineStr"/>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>AI remarks unavailable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-08-14 10:19:04 IST</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Loser</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>REGENCERAM</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Regency Ceramics Limited</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>37</v>
+      </c>
+      <c r="F35" t="n">
+        <v>43.99</v>
+      </c>
+      <c r="G35" t="n">
+        <v>43.99</v>
+      </c>
+      <c r="H35" t="n">
+        <v>36.31</v>
+      </c>
+      <c r="I35" t="n">
+        <v>40.33</v>
+      </c>
+      <c r="J35" t="n">
+        <v>37</v>
+      </c>
+      <c r="K35" t="n">
+        <v>19032</v>
+      </c>
+      <c r="L35" t="n">
+        <v>-8.26</v>
+      </c>
+      <c r="M35" t="inlineStr"/>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>AI remarks unavailable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-08-14 10:19:04 IST</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Loser</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>ASIANENE</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Asian Energy Services Limited</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>375.2</v>
+      </c>
+      <c r="F36" t="n">
+        <v>399</v>
+      </c>
+      <c r="G36" t="n">
+        <v>399</v>
+      </c>
+      <c r="H36" t="n">
+        <v>370.75</v>
+      </c>
+      <c r="I36" t="n">
+        <v>410</v>
+      </c>
+      <c r="J36" t="n">
+        <v>375.2</v>
+      </c>
+      <c r="K36" t="n">
+        <v>471071</v>
+      </c>
+      <c r="L36" t="n">
+        <v>-8.49</v>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>Asian Energy Services Files June-Quarter Unaudited Results with SEBI - tipranks.com</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>['Asian Energy Services Files June-Quarter Unaudited Results with SEBI - tipranks.com', 'Asian Energy Services secures ₹131.39 crore from convertible warrants - Business Upturn']</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>AI remarks unavailable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-08-14 10:19:04 IST</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Loser</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>TARMAT</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Tarmat Limited</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>59.11</v>
+      </c>
+      <c r="F37" t="n">
+        <v>68.5</v>
+      </c>
+      <c r="G37" t="n">
+        <v>69.65000000000001</v>
+      </c>
+      <c r="H37" t="n">
+        <v>57.44</v>
+      </c>
+      <c r="I37" t="n">
+        <v>64.68000000000001</v>
+      </c>
+      <c r="J37" t="n">
+        <v>59.11</v>
+      </c>
+      <c r="K37" t="n">
+        <v>506108</v>
+      </c>
+      <c r="L37" t="n">
+        <v>-8.609999999999999</v>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>Tarmat Ltd. Share Price News: Price Action, Fundamentals - Univest</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>['Tarmat Ltd. Share Price News: Price Action, Fundamentals - Univest', 'Tarmat Ltd announces demise of promoter group member holding 4.19% stake - scanx.trade']</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>AI remarks unavailable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-08-14 10:19:04 IST</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Loser</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>ABMINTLLTD</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>ABM International Limited</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>62.44</v>
+      </c>
+      <c r="F38" t="n">
+        <v>72.8</v>
+      </c>
+      <c r="G38" t="n">
+        <v>72.8</v>
+      </c>
+      <c r="H38" t="n">
+        <v>62.44</v>
+      </c>
+      <c r="I38" t="n">
+        <v>69.37</v>
+      </c>
+      <c r="J38" t="n">
+        <v>62.44</v>
+      </c>
+      <c r="K38" t="n">
+        <v>20529</v>
+      </c>
+      <c r="L38" t="n">
+        <v>-9.99</v>
+      </c>
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>AI remarks unavailable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-08-14 10:19:04 IST</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Loser</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>COCKERILL</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>John Cockerill India Limited</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>8418</v>
+      </c>
+      <c r="F39" t="n">
+        <v>8624</v>
+      </c>
+      <c r="G39" t="n">
+        <v>9040</v>
+      </c>
+      <c r="H39" t="n">
+        <v>8380</v>
+      </c>
+      <c r="I39" t="n">
+        <v>10101.5</v>
+      </c>
+      <c r="J39" t="n">
+        <v>8418</v>
+      </c>
+      <c r="K39" t="n">
+        <v>62941</v>
+      </c>
+      <c r="L39" t="n">
+        <v>-16.67</v>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>Earnings call transcript: John Cockerill India Q2 2026 revenue jumps, stock rises 4.7% - Investing.com</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>['Earnings call transcript: John Cockerill India Q2 2026 revenue jumps, stock rises 4.7% - Investing.com', 'COCKERILL: Strong revenue growth and robust order backlog drive improved profitability and future outlook - TradingView', 'John Cockerill India reports standalone net loss of Rs 4.58 crore in the June 2026 quarter - business-standard.com', 'John Cockerill India Limited Announces Cessation of Marc Dumont as Key Managerial Personnel, Effective July 31, 2026 - marketscreener.com', 'John Cockerill India Q2 2026 slides: 82% revenue surge, INR 4,600cr backlog - Investing.com']</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>AI remarks unavailable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-08-14 10:19:04 IST</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Loser</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>SHANTI-RE</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Shanti Gold International Limited-RE</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>14</v>
+      </c>
+      <c r="F40" t="n">
+        <v>18</v>
+      </c>
+      <c r="G40" t="n">
+        <v>18</v>
+      </c>
+      <c r="H40" t="n">
+        <v>11.05</v>
+      </c>
+      <c r="I40" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="J40" t="n">
+        <v>14</v>
+      </c>
+      <c r="K40" t="n">
+        <v>58494</v>
+      </c>
+      <c r="L40" t="n">
+        <v>-17.16</v>
+      </c>
+      <c r="M40" t="inlineStr"/>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>AI remarks unavailable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-08-14 10:19:04 IST</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Loser</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>GENESYS-RE</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Genesys International Corporation Limited-RE</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>128.1</v>
+      </c>
+      <c r="F41" t="n">
+        <v>141</v>
+      </c>
+      <c r="G41" t="n">
+        <v>141</v>
+      </c>
+      <c r="H41" t="n">
+        <v>115.6</v>
+      </c>
+      <c r="I41" t="n">
+        <v>161.3</v>
+      </c>
+      <c r="J41" t="n">
+        <v>128.1</v>
+      </c>
+      <c r="K41" t="n">
+        <v>505071</v>
+      </c>
+      <c r="L41" t="n">
+        <v>-20.58</v>
+      </c>
+      <c r="M41" t="inlineStr"/>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>AI remarks unavailable.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O21"/>
+  <autoFilter ref="A1:O41"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>